<commit_message>
Publish complete IPS report packs with verified recovery controls
</commit_message>
<xml_diff>
--- a/output/investment_committee_report.xlsx
+++ b/output/investment_committee_report.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Constraint Validation'!$A$1:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Methodology'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Data Provenance'!$A$1:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Source Summary'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Source Summary'!$A$1:$M$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21802,7 +21802,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\efficient_frontier.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\recommended_allocation.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\cumulative_performance_vs_benchmark.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\drawdown_comparison.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\factor_exposures.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\equity_sleeve_factor_exposures.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\risk_contribution.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\policy_drift.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\stress_test_results.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\rolling_return.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\rolling_volatility.png; C:\Users\perso\Documents\GitHub\ips-driven-asset-allocation-engine\charts\rolling_drawdown.png</t>
+          <t>charts\efficient_frontier.png; charts\recommended_allocation.png; charts\cumulative_performance_vs_benchmark.png; charts\drawdown_comparison.png; charts\factor_exposures.png; charts\equity_sleeve_factor_exposures.png; charts\risk_contribution.png; charts\policy_drift.png; charts\stress_test_results.png; charts\rolling_return.png; charts\rolling_volatility.png; charts\rolling_drawdown.png</t>
         </is>
       </c>
     </row>
@@ -22293,18 +22293,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -22320,37 +22324,57 @@
       </c>
       <c r="C1" s="19" t="inlineStr">
         <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="D1" s="19" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="E1" s="19" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="F1" s="19" t="inlineStr">
+        <is>
           <t>monthly_returns_sha256</t>
         </is>
       </c>
-      <c r="D1" s="19" t="inlineStr">
+      <c r="G1" s="19" t="inlineStr">
         <is>
           <t>complete_months</t>
         </is>
       </c>
-      <c r="E1" s="19" t="inlineStr">
+      <c r="H1" s="19" t="inlineStr">
         <is>
           <t>mode</t>
         </is>
       </c>
-      <c r="F1" s="19" t="inlineStr">
+      <c r="I1" s="19" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="G1" s="19" t="inlineStr">
+      <c r="J1" s="19" t="inlineStr">
         <is>
           <t>source_reference</t>
         </is>
       </c>
-      <c r="H1" s="19" t="inlineStr">
+      <c r="K1" s="19" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="I1" s="19" t="inlineStr">
+      <c r="L1" s="19" t="inlineStr">
         <is>
           <t>factor_data_sha256</t>
+        </is>
+      </c>
+      <c r="M1" s="19" t="inlineStr">
+        <is>
+          <t>requested_end</t>
         </is>
       </c>
     </row>
@@ -22367,17 +22391,33 @@
       </c>
       <c r="C2" s="24" t="inlineStr">
         <is>
+          <t>6dcc8d9852ce4a228f2e6607227bf609</t>
+        </is>
+      </c>
+      <c r="D2" s="24" t="inlineStr">
+        <is>
+          <t>2015-06-30</t>
+        </is>
+      </c>
+      <c r="E2" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="F2" s="24" t="inlineStr">
+        <is>
           <t>21ef359c814c516f99b2af719280741dde5d858a92fac4df608b97630f211c8c</t>
         </is>
       </c>
-      <c r="D2" s="24" t="n">
+      <c r="G2" s="24" t="n">
         <v>132</v>
       </c>
-      <c r="E2" s="24" t="inlineStr"/>
-      <c r="F2" s="24" t="inlineStr"/>
-      <c r="G2" s="24" t="inlineStr"/>
       <c r="H2" s="24" t="inlineStr"/>
       <c r="I2" s="24" t="inlineStr"/>
+      <c r="J2" s="24" t="inlineStr"/>
+      <c r="K2" s="24" t="inlineStr"/>
+      <c r="L2" s="24" t="inlineStr"/>
+      <c r="M2" s="24" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
@@ -22392,29 +22432,33 @@
       </c>
       <c r="C3" s="24" t="inlineStr"/>
       <c r="D3" s="24" t="inlineStr"/>
-      <c r="E3" s="24" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr"/>
+      <c r="F3" s="24" t="inlineStr"/>
+      <c r="G3" s="24" t="inlineStr"/>
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>synthetic</t>
         </is>
       </c>
-      <c r="F3" s="24" t="inlineStr">
+      <c r="I3" s="24" t="inlineStr">
         <is>
           <t>Deterministic synthetic factor generator</t>
         </is>
       </c>
-      <c r="G3" s="24" t="inlineStr">
+      <c r="J3" s="24" t="inlineStr">
         <is>
           <t>src/factor_model.py::generate_fallback_factors</t>
         </is>
       </c>
-      <c r="H3" s="24" t="n">
+      <c r="K3" s="24" t="n">
         <v>49</v>
       </c>
-      <c r="I3" s="24" t="inlineStr">
+      <c r="L3" s="24" t="inlineStr">
         <is>
           <t>e154e0794d3a3a8569f74780b8ff49df79bebcb4b302a5062668c9e4a99d0fe6</t>
         </is>
       </c>
+      <c r="M3" s="24" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -22434,9 +22478,48 @@
       <c r="G4" s="24" t="inlineStr"/>
       <c r="H4" s="24" t="inlineStr"/>
       <c r="I4" s="24" t="inlineStr"/>
+      <c r="J4" s="24" t="inlineStr"/>
+      <c r="K4" s="24" t="inlineStr"/>
+      <c r="L4" s="24" t="inlineStr"/>
+      <c r="M4" s="24" t="inlineStr"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr"/>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>6dcc8d9852ce4a228f2e6607227bf609</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>2015-06-30</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr"/>
+      <c r="G5" s="24" t="inlineStr"/>
+      <c r="H5" s="24" t="inlineStr"/>
+      <c r="I5" s="24" t="inlineStr"/>
+      <c r="J5" s="24" t="inlineStr"/>
+      <c r="K5" s="24" t="inlineStr"/>
+      <c r="L5" s="24" t="inlineStr"/>
+      <c r="M5" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
+  <autoFilter ref="A1:M5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>